<commit_message>
Add two Tewogbola et al. (2025) Nigeria HPT preprints
Tewogbola2025-ins: Health Insurance Purchase Task, Nigeria (N=106).
First African-country entry -- introduces "Nigeria" and "Africa" as
country/region values.

Tewogbola2025-mil: HPT-style demand curve applied to support for U.S.
military intervention, with likelihood of success substituted for
monetary price. Not a purchase/consumption commodity like everything
else in the index -- included per the About page's stated allowance
for non-monetary price substitutes, but flagged in its own notes as
the furthest stretch of "commodity" coded so far.

Both are self-authored PROMISE Labs Africa preprints (medRxiv, SSRN),
not yet peer-reviewed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL372"/>
+  <dimension ref="A1:AL374"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -72047,8 +72047,337 @@
         </is>
       </c>
     </row>
-    <row r="373" ht="13" customHeight="1"/>
-    <row r="374" ht="13" customHeight="1"/>
+    <row r="373" ht="13" customHeight="1">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-ins</t>
+        </is>
+      </c>
+      <c r="B373" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>medRxiv (preprint)</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>10.1101/2025.08.27.25334236</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>https://www.medrxiv.org/content/10.1101/2025.08.27.25334236v1</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>Health insurance</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N373" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="O373" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="P373" t="n">
+        <v>106</v>
+      </c>
+      <c r="Q373" t="inlineStr">
+        <is>
+          <t>General community sample (Nigerian adults)</t>
+        </is>
+      </c>
+      <c r="R373" t="n">
+        <v>29.48</v>
+      </c>
+      <c r="S373" t="n">
+        <v>15</v>
+      </c>
+      <c r="T373" t="n">
+        <v>5</v>
+      </c>
+      <c r="U373" t="n">
+        <v>560000</v>
+      </c>
+      <c r="V373" t="inlineStr">
+        <is>
+          <t>NGN</t>
+        </is>
+      </c>
+      <c r="W373" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X373" t="inlineStr">
+        <is>
+          <t>Empirical</t>
+        </is>
+      </c>
+      <c r="Y373" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z373" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA373" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB373" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC373" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD373" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE373" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AF373" t="inlineStr">
+        <is>
+          <t>AUC (used as individual-level demand proxy; Q0/alpha could not be fit per-individual on dichotomous Yes/No responses)</t>
+        </is>
+      </c>
+      <c r="AG373" t="n">
+        <v>6.3e-05</v>
+      </c>
+      <c r="AH373" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="AJ373" t="n">
+        <v>18478.78</v>
+      </c>
+      <c r="AK373" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="AL373" t="inlineStr">
+        <is>
+          <t>Preprint, self-authored by the PI (PROMISE Labs Africa). Aggregate exponential/exponentiated demand model fit to pooled Yes/No purchase responses across all 106 participants (Figure 1); individual-level Q0/alpha could not be estimated from dichotomous responses, so a normalized AUC was used as an individual-level proxy instead. Values here are the full-sample aggregate model, not the open/closed-economy subgroup splits reported separately in the paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="374" ht="13" customHeight="1">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-mil</t>
+        </is>
+      </c>
+      <c r="B374" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>SSRN (preprint)</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>10.2139/ssrn.7167500</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=7167500</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>Support for U.S. military intervention</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>Cross-sectional</t>
+        </is>
+      </c>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N374" t="inlineStr">
+        <is>
+          <t>Nigeria</t>
+        </is>
+      </c>
+      <c r="O374" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="P374" t="n">
+        <v>106</v>
+      </c>
+      <c r="Q374" t="inlineStr">
+        <is>
+          <t>General community sample (Nigerian adults)</t>
+        </is>
+      </c>
+      <c r="R374" t="n">
+        <v>30.03</v>
+      </c>
+      <c r="S374" t="n">
+        <v>10</v>
+      </c>
+      <c r="T374" t="n">
+        <v>0</v>
+      </c>
+      <c r="U374" t="n">
+        <v>100</v>
+      </c>
+      <c r="V374" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W374" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X374" t="inlineStr">
+        <is>
+          <t>Empirical</t>
+        </is>
+      </c>
+      <c r="Y374" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z374" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA374" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB374" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC374" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AD374" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE374" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AF374" t="inlineStr">
+        <is>
+          <t>P50 = 16.87% (likelihood of success at which the fitted model predicts 50% support)</t>
+        </is>
+      </c>
+      <c r="AG374" t="n">
+        <v>0.000155</v>
+      </c>
+      <c r="AH374" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="AK374" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="AL374" t="inlineStr">
+        <is>
+          <t>Preprint, self-authored by the PI (PROMISE Labs Africa). Not a purchase/consumption commodity -- an HPT-style demand curve applied to policy support, with likelihood of successful violence suppression (100%-0%) substituted for monetary price (modeled as odds against success). lowest_price/highest_price above represent that 0-100% likelihood scale, not currency. Included per the site's stated scope allowance for non-monetary price substitutes, but it is the furthest stretch of "commodity" in the index so far -- flagged for reconsideration if that scope guidance changes. Values are the full-sample aggregate model (N=106), not the demographic subgroup splits reported separately in the paper.</t>
+        </is>
+      </c>
+    </row>
     <row r="375" ht="13" customHeight="1"/>
     <row r="376" ht="13" customHeight="1"/>
     <row r="377" ht="13" customHeight="1"/>

</xml_diff>

<commit_message>
Correct Tewogbola2025-ins sample size to N=78
Table 1 reports N=106 for most participant characteristics, but the
experimental condition itself (Economy Type Assigned To) and
Household Income both sum to only 78 with the other 28 unaccounted
for. 78 is the sample actually analyzable on the condition the demand
curve is split by. Noted in-record that this is a preprint still
under peer review and may be revised on acceptance.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -72122,7 +72122,7 @@
         </is>
       </c>
       <c r="P373" t="n">
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="Q373" t="inlineStr">
         <is>
@@ -72210,7 +72210,7 @@
       </c>
       <c r="AL373" t="inlineStr">
         <is>
-          <t>Preprint, self-authored by the PI (PROMISE Labs Africa). Aggregate exponential/exponentiated demand model fit to pooled Yes/No purchase responses across all 106 participants (Figure 1); individual-level Q0/alpha could not be estimated from dichotomous responses, so a normalized AUC was used as an individual-level proxy instead. Values here are the full-sample aggregate model, not the open/closed-economy subgroup splits reported separately in the paper.</t>
+          <t>Preprint, self-authored by the PI (PROMISE Labs Africa); still under peer review, sample size may be revised once a final accepted version exists. N=78 used here (not the N=106 total recruited) -- Table 1 reports 106 for most characteristics, but Economy Type Assigned To (the experimental condition the demand analysis is split on) and Household Income both sum to only 78 with no accounting for the other 28, so 78 is treated as the analyzed sample. Aggregate exponential/exponentiated demand model fit to pooled Yes/No purchase responses (Figure 1); individual-level Q0/alpha could not be estimated from dichotomous responses, so a normalized AUC was used as an individual-level proxy instead. Values here are the full-sample aggregate model, not the open/closed-economy subgroup splits reported separately in the paper.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Goto et al. (2026) theft recidivism/kleptomania HPT (3 rows)
Independent Japan-based group, bioRxiv preprint, not yet peer-
reviewed. Three-group study (control, theft recidivists with/without
kleptomania) coded as 3 rows since the groups aren't meaningfully
poolable -- the study's point is the group difference. First Japan/
JPY/Asia entries in the index.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL374"/>
+  <dimension ref="A1:AL377"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -72378,9 +72378,498 @@
         </is>
       </c>
     </row>
-    <row r="375" ht="13" customHeight="1"/>
-    <row r="376" ht="13" customHeight="1"/>
-    <row r="377" ht="13" customHeight="1"/>
+    <row r="375" ht="13" customHeight="1">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Goto2026-ct</t>
+        </is>
+      </c>
+      <c r="B375" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>bioRxiv (preprint)</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>10.64898/2026.07.26.740843</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.07.26.740843</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>Snack food</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Food &amp; Nutrition</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>Cross-sectional</t>
+        </is>
+      </c>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N375" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="O375" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="P375" t="n">
+        <v>52</v>
+      </c>
+      <c r="Q375" t="inlineStr">
+        <is>
+          <t>General community sample (no criminal record)</t>
+        </is>
+      </c>
+      <c r="S375" t="n">
+        <v>9</v>
+      </c>
+      <c r="T375" t="n">
+        <v>0</v>
+      </c>
+      <c r="U375" t="n">
+        <v>5000</v>
+      </c>
+      <c r="V375" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="W375" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="X375" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y375" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z375" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA375" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB375" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC375" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD375" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE375" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AF375" t="inlineStr">
+        <is>
+          <t>Omax (maximum expenditure)</t>
+        </is>
+      </c>
+      <c r="AG375" t="n">
+        <v>0.446</v>
+      </c>
+      <c r="AH375" t="n">
+        <v>20.66</v>
+      </c>
+      <c r="AI375" t="n">
+        <v>1740</v>
+      </c>
+      <c r="AJ375" t="n">
+        <v>348.9</v>
+      </c>
+      <c r="AL375" t="inlineStr">
+        <is>
+          <t>Not self-authored -- independent Japan-based group (Kyoto University et al.), bioRxiv preprint, not yet peer-reviewed. Three-group study (theft recidivists with/without kleptomania vs. healthy controls); coded as 3 rows since averaging clinical and control groups would misrepresent the finding (the study's point is the group difference), same pattern used for multi-commodity papers split by commodity. Commodity is a self-nominated favorite snack/sweet (not a fixed item), coded as "Snack food". Demand model equation not stated in the main text (paper reports indices Q0, alpha, Omax, Pmax, breakpoint without citing a specific curve-fitting equation); R2 not reported anywhere. Mean age not broken out by group in the main text (only a combined TR-vs-CT test was reported: not significantly different). Also administered a balloon analogue risk task (BART) with fNIRS measurement of prefrontal cortex activity -- out of HPT scope, not coded here. First Japan/JPY/Asia entries in the index. This row: control (CT) group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="376" ht="13" customHeight="1">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Goto2026-trnk</t>
+        </is>
+      </c>
+      <c r="B376" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>bioRxiv (preprint)</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>10.64898/2026.07.26.740843</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.07.26.740843</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>Snack food</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Food &amp; Nutrition</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>Cross-sectional</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N376" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="O376" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="P376" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q376" t="inlineStr">
+        <is>
+          <t>Theft recidivists without kleptomania</t>
+        </is>
+      </c>
+      <c r="S376" t="n">
+        <v>9</v>
+      </c>
+      <c r="T376" t="n">
+        <v>0</v>
+      </c>
+      <c r="U376" t="n">
+        <v>5000</v>
+      </c>
+      <c r="V376" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="W376" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="X376" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA376" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD376" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE376" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AF376" t="inlineStr">
+        <is>
+          <t>Omax (maximum expenditure)</t>
+        </is>
+      </c>
+      <c r="AG376" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="AH376" t="n">
+        <v>76.34999999999999</v>
+      </c>
+      <c r="AI376" t="n">
+        <v>1694</v>
+      </c>
+      <c r="AJ376" t="n">
+        <v>293.8</v>
+      </c>
+      <c r="AL376" t="inlineStr">
+        <is>
+          <t>Not self-authored -- independent Japan-based group (Kyoto University et al.), bioRxiv preprint, not yet peer-reviewed. Three-group study (theft recidivists with/without kleptomania vs. healthy controls); coded as 3 rows since averaging clinical and control groups would misrepresent the finding (the study's point is the group difference), same pattern used for multi-commodity papers split by commodity. Commodity is a self-nominated favorite snack/sweet (not a fixed item), coded as "Snack food". Demand model equation not stated in the main text (paper reports indices Q0, alpha, Omax, Pmax, breakpoint without citing a specific curve-fitting equation); R2 not reported anywhere. Mean age not broken out by group in the main text (only a combined TR-vs-CT test was reported: not significantly different). Also administered a balloon analogue risk task (BART) with fNIRS measurement of prefrontal cortex activity -- out of HPT scope, not coded here. First Japan/JPY/Asia entries in the index. This row: theft recidivists without kleptomania (TR-NK).</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" ht="13" customHeight="1">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Goto2026-trka</t>
+        </is>
+      </c>
+      <c r="B377" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>bioRxiv (preprint)</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>10.64898/2026.07.26.740843</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.64898/2026.07.26.740843</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>Snack food</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Food &amp; Nutrition</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>Cross-sectional</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N377" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="P377" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q377" t="inlineStr">
+        <is>
+          <t>Theft recidivists with kleptomania</t>
+        </is>
+      </c>
+      <c r="S377" t="n">
+        <v>9</v>
+      </c>
+      <c r="T377" t="n">
+        <v>0</v>
+      </c>
+      <c r="U377" t="n">
+        <v>5000</v>
+      </c>
+      <c r="V377" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="W377" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="X377" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA377" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD377" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE377" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AF377" t="inlineStr">
+        <is>
+          <t>Omax (maximum expenditure)</t>
+        </is>
+      </c>
+      <c r="AG377" t="n">
+        <v>0.601</v>
+      </c>
+      <c r="AH377" t="n">
+        <v>112.3</v>
+      </c>
+      <c r="AI377" t="n">
+        <v>1838</v>
+      </c>
+      <c r="AJ377" t="n">
+        <v>124.9</v>
+      </c>
+      <c r="AL377" t="inlineStr">
+        <is>
+          <t>Not self-authored -- independent Japan-based group (Kyoto University et al.), bioRxiv preprint, not yet peer-reviewed. Three-group study (theft recidivists with/without kleptomania vs. healthy controls); coded as 3 rows since averaging clinical and control groups would misrepresent the finding (the study's point is the group difference), same pattern used for multi-commodity papers split by commodity. Commodity is a self-nominated favorite snack/sweet (not a fixed item), coded as "Snack food". Demand model equation not stated in the main text (paper reports indices Q0, alpha, Omax, Pmax, breakpoint without citing a specific curve-fitting equation); R2 not reported anywhere. Mean age not broken out by group in the main text (only a combined TR-vs-CT test was reported: not significantly different). Also administered a balloon analogue risk task (BART) with fNIRS measurement of prefrontal cortex activity -- out of HPT scope, not coded here. First Japan/JPY/Asia entries in the index. This row: theft recidivists with kleptomania (TR-KA).</t>
+        </is>
+      </c>
+    </row>
     <row r="378" ht="13" customHeight="1"/>
     <row r="379" ht="13" customHeight="1"/>
     <row r="380" ht="13" customHeight="1"/>

</xml_diff>

<commit_message>
Collapse Goto2026 3 rows into 1: N summed, BE indices averaged
Per request: single row instead of one-per-population. N = 52+40+16 =
108; Q0/alpha/Pmax/breakpoint = simple (unweighted) mean across the 3
groups. Notes flag that this obscures the paper's actual finding
(the kleptomania group differed sharply from the other two) and
point back to the source paper for the real per-group values.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL377"/>
+  <dimension ref="A1:AL375"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -72381,7 +72381,7 @@
     <row r="375" ht="13" customHeight="1">
       <c r="A375" t="inlineStr">
         <is>
-          <t>Goto2026-ct</t>
+          <t>Goto2026</t>
         </is>
       </c>
       <c r="B375" t="n">
@@ -72453,11 +72453,11 @@
         </is>
       </c>
       <c r="P375" t="n">
-        <v>52</v>
+        <v>108</v>
       </c>
       <c r="Q375" t="inlineStr">
         <is>
-          <t>General community sample (no criminal record)</t>
+          <t>Combined: control subjects with no criminal record, theft recidivists without kleptomania, and theft recidivists with kleptomania</t>
         </is>
       </c>
       <c r="S375" t="n">
@@ -72525,351 +72525,25 @@
         </is>
       </c>
       <c r="AG375" t="n">
-        <v>0.446</v>
+        <v>0.487</v>
       </c>
       <c r="AH375" t="n">
-        <v>20.66</v>
+        <v>69.77</v>
       </c>
       <c r="AI375" t="n">
-        <v>1740</v>
+        <v>1757.33</v>
       </c>
       <c r="AJ375" t="n">
-        <v>348.9</v>
+        <v>255.87</v>
       </c>
       <c r="AL375" t="inlineStr">
         <is>
-          <t>Not self-authored -- independent Japan-based group (Kyoto University et al.), bioRxiv preprint, not yet peer-reviewed. Three-group study (theft recidivists with/without kleptomania vs. healthy controls); coded as 3 rows since averaging clinical and control groups would misrepresent the finding (the study's point is the group difference), same pattern used for multi-commodity papers split by commodity. Commodity is a self-nominated favorite snack/sweet (not a fixed item), coded as "Snack food". Demand model equation not stated in the main text (paper reports indices Q0, alpha, Omax, Pmax, breakpoint without citing a specific curve-fitting equation); R2 not reported anywhere. Mean age not broken out by group in the main text (only a combined TR-vs-CT test was reported: not significantly different). Also administered a balloon analogue risk task (BART) with fNIRS measurement of prefrontal cortex activity -- out of HPT scope, not coded here. First Japan/JPY/Asia entries in the index. This row: control (CT) group.</t>
+          <t>Not self-authored -- independent Japan-based group (Kyoto University et al.), bioRxiv preprint, not yet peer-reviewed. Original paper reports 3 separate populations (control N=52, theft recidivists without kleptomania N=40, theft recidivists with kleptomania N=16) with distinct Q0/alpha/Omax/Pmax/breakpoint per group -- collapsed here into one row: N summed (108), indices averaged (simple mean across the 3 groups, not N-weighted). This obscures the paper's actual finding, which is the group difference (kleptomania group showed markedly higher Q0, alpha, and breakpoint than the other two) -- see the paper directly for the real per-group values. Commodity is a self-nominated favorite snack/sweet (not a fixed item), coded as "Snack food". Demand model equation not stated in the main text; R2 not reported. Mean age not broken out by group. Also administered a balloon analogue risk task (BART) with fNIRS measurement of prefrontal cortex activity -- out of HPT scope, not coded here. First Japan/JPY/Asia entries in the index.</t>
         </is>
       </c>
     </row>
-    <row r="376" ht="13" customHeight="1">
-      <c r="A376" t="inlineStr">
-        <is>
-          <t>Goto2026-trnk</t>
-        </is>
-      </c>
-      <c r="B376" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C376" t="inlineStr">
-        <is>
-          <t>bioRxiv (preprint)</t>
-        </is>
-      </c>
-      <c r="D376" t="inlineStr">
-        <is>
-          <t>10.64898/2026.07.26.740843</t>
-        </is>
-      </c>
-      <c r="E376" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.64898/2026.07.26.740843</t>
-        </is>
-      </c>
-      <c r="F376" t="inlineStr">
-        <is>
-          <t>Preprint</t>
-        </is>
-      </c>
-      <c r="G376" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H376" t="inlineStr">
-        <is>
-          <t>Snack food</t>
-        </is>
-      </c>
-      <c r="I376" t="inlineStr">
-        <is>
-          <t>Food &amp; Nutrition</t>
-        </is>
-      </c>
-      <c r="J376" t="inlineStr">
-        <is>
-          <t>Cross-sectional</t>
-        </is>
-      </c>
-      <c r="K376" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="L376" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M376" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N376" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="O376" t="inlineStr">
-        <is>
-          <t>Asia</t>
-        </is>
-      </c>
-      <c r="P376" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q376" t="inlineStr">
-        <is>
-          <t>Theft recidivists without kleptomania</t>
-        </is>
-      </c>
-      <c r="S376" t="n">
-        <v>9</v>
-      </c>
-      <c r="T376" t="n">
-        <v>0</v>
-      </c>
-      <c r="U376" t="n">
-        <v>5000</v>
-      </c>
-      <c r="V376" t="inlineStr">
-        <is>
-          <t>JPY</t>
-        </is>
-      </c>
-      <c r="W376" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="X376" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="Y376" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Z376" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="AA376" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AB376" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="AC376" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="AD376" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AE376" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AF376" t="inlineStr">
-        <is>
-          <t>Omax (maximum expenditure)</t>
-        </is>
-      </c>
-      <c r="AG376" t="n">
-        <v>0.414</v>
-      </c>
-      <c r="AH376" t="n">
-        <v>76.34999999999999</v>
-      </c>
-      <c r="AI376" t="n">
-        <v>1694</v>
-      </c>
-      <c r="AJ376" t="n">
-        <v>293.8</v>
-      </c>
-      <c r="AL376" t="inlineStr">
-        <is>
-          <t>Not self-authored -- independent Japan-based group (Kyoto University et al.), bioRxiv preprint, not yet peer-reviewed. Three-group study (theft recidivists with/without kleptomania vs. healthy controls); coded as 3 rows since averaging clinical and control groups would misrepresent the finding (the study's point is the group difference), same pattern used for multi-commodity papers split by commodity. Commodity is a self-nominated favorite snack/sweet (not a fixed item), coded as "Snack food". Demand model equation not stated in the main text (paper reports indices Q0, alpha, Omax, Pmax, breakpoint without citing a specific curve-fitting equation); R2 not reported anywhere. Mean age not broken out by group in the main text (only a combined TR-vs-CT test was reported: not significantly different). Also administered a balloon analogue risk task (BART) with fNIRS measurement of prefrontal cortex activity -- out of HPT scope, not coded here. First Japan/JPY/Asia entries in the index. This row: theft recidivists without kleptomania (TR-NK).</t>
-        </is>
-      </c>
-    </row>
-    <row r="377" ht="13" customHeight="1">
-      <c r="A377" t="inlineStr">
-        <is>
-          <t>Goto2026-trka</t>
-        </is>
-      </c>
-      <c r="B377" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C377" t="inlineStr">
-        <is>
-          <t>bioRxiv (preprint)</t>
-        </is>
-      </c>
-      <c r="D377" t="inlineStr">
-        <is>
-          <t>10.64898/2026.07.26.740843</t>
-        </is>
-      </c>
-      <c r="E377" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.64898/2026.07.26.740843</t>
-        </is>
-      </c>
-      <c r="F377" t="inlineStr">
-        <is>
-          <t>Preprint</t>
-        </is>
-      </c>
-      <c r="G377" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H377" t="inlineStr">
-        <is>
-          <t>Snack food</t>
-        </is>
-      </c>
-      <c r="I377" t="inlineStr">
-        <is>
-          <t>Food &amp; Nutrition</t>
-        </is>
-      </c>
-      <c r="J377" t="inlineStr">
-        <is>
-          <t>Cross-sectional</t>
-        </is>
-      </c>
-      <c r="K377" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="L377" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M377" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N377" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="O377" t="inlineStr">
-        <is>
-          <t>Asia</t>
-        </is>
-      </c>
-      <c r="P377" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q377" t="inlineStr">
-        <is>
-          <t>Theft recidivists with kleptomania</t>
-        </is>
-      </c>
-      <c r="S377" t="n">
-        <v>9</v>
-      </c>
-      <c r="T377" t="n">
-        <v>0</v>
-      </c>
-      <c r="U377" t="n">
-        <v>5000</v>
-      </c>
-      <c r="V377" t="inlineStr">
-        <is>
-          <t>JPY</t>
-        </is>
-      </c>
-      <c r="W377" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="X377" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="Y377" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="Z377" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="AA377" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="AB377" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="AC377" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="AD377" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AE377" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="AF377" t="inlineStr">
-        <is>
-          <t>Omax (maximum expenditure)</t>
-        </is>
-      </c>
-      <c r="AG377" t="n">
-        <v>0.601</v>
-      </c>
-      <c r="AH377" t="n">
-        <v>112.3</v>
-      </c>
-      <c r="AI377" t="n">
-        <v>1838</v>
-      </c>
-      <c r="AJ377" t="n">
-        <v>124.9</v>
-      </c>
-      <c r="AL377" t="inlineStr">
-        <is>
-          <t>Not self-authored -- independent Japan-based group (Kyoto University et al.), bioRxiv preprint, not yet peer-reviewed. Three-group study (theft recidivists with/without kleptomania vs. healthy controls); coded as 3 rows since averaging clinical and control groups would misrepresent the finding (the study's point is the group difference), same pattern used for multi-commodity papers split by commodity. Commodity is a self-nominated favorite snack/sweet (not a fixed item), coded as "Snack food". Demand model equation not stated in the main text (paper reports indices Q0, alpha, Omax, Pmax, breakpoint without citing a specific curve-fitting equation); R2 not reported anywhere. Mean age not broken out by group in the main text (only a combined TR-vs-CT test was reported: not significantly different). Also administered a balloon analogue risk task (BART) with fNIRS measurement of prefrontal cortex activity -- out of HPT scope, not coded here. First Japan/JPY/Asia entries in the index. This row: theft recidivists with kleptomania (TR-KA).</t>
-        </is>
-      </c>
-    </row>
+    <row r="376" ht="13" customHeight="1"/>
+    <row r="377" ht="13" customHeight="1"/>
     <row r="378" ht="13" customHeight="1"/>
     <row r="379" ht="13" customHeight="1"/>
     <row r="380" ht="13" customHeight="1"/>

</xml_diff>

<commit_message>
Add Yang et al. (2024) China cigarette purchase task study
Peer-reviewed (Journal of Peking University Health Sciences), not a
preprint. Baseline data from a smoking-cessation trial, N=447 male
smokers. First China/CNY entry. First entry with an explicitly
reported k value (1.201) rather than "Empirical".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL375"/>
+  <dimension ref="A1:AL376"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -72542,7 +72542,177 @@
         </is>
       </c>
     </row>
-    <row r="376" ht="13" customHeight="1"/>
+    <row r="376" ht="13" customHeight="1">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Yang2024</t>
+        </is>
+      </c>
+      <c r="B376" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Journal of Peking University (Health Sciences)</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>10.19723/j.issn.1671-167X.2024.03.015</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.19723/j.issn.1671-167X.2024.03.015</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>Cigarettes</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Tobacco &amp; Nicotine</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>Secondary analysis</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N376" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="O376" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="P376" t="n">
+        <v>447</v>
+      </c>
+      <c r="Q376" t="inlineStr">
+        <is>
+          <t>Adult male smokers (coal mining/manufacturing/energy industries; Jiangsu, Inner Mongolia, Hebei)</t>
+        </is>
+      </c>
+      <c r="R376" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="S376" t="n">
+        <v>13</v>
+      </c>
+      <c r="T376" t="n">
+        <v>0</v>
+      </c>
+      <c r="U376" t="n">
+        <v>600</v>
+      </c>
+      <c r="V376" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="W376" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X376" t="n">
+        <v>1.201</v>
+      </c>
+      <c r="Y376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC376" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD376" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE376" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AF376" t="inlineStr">
+        <is>
+          <t>Omax (maximum expenditure)</t>
+        </is>
+      </c>
+      <c r="AG376" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AH376" t="inlineStr">
+        <is>
+          <t>20 (median)</t>
+        </is>
+      </c>
+      <c r="AI376" t="inlineStr">
+        <is>
+          <t>180 (median)</t>
+        </is>
+      </c>
+      <c r="AJ376" t="inlineStr">
+        <is>
+          <t>60 (median)</t>
+        </is>
+      </c>
+      <c r="AL376" t="inlineStr">
+        <is>
+          <t>Peer-reviewed journal article (Journal of Peking University Health Sciences), not a preprint. Data are baseline responses from a prospective smoking-cessation intervention trial (504 recruited -&gt; 451 valid after removing 53 non-systematic cases -&gt; 447 after excluding 4 non-converging individual fits). All participants male (recruited from coal mining/machinery manufacturing/energy industries in Jiangsu, Inner Mongolia, and Hebei provinces), so no gender reported. Q0/breakpoint/Omax/Pmax in Table 1 are medians (IQR), not means -- reported as such here. Two elasticity figures given: an individual-level log-transformed mean (-2.21 +/- 0.53 SD) and a back-transformed aggregate value (0.54) used for the paper's own smoking-cessation-rate policy simulation; mean_alpha here uses the latter (0.54), consistent with the non-log alpha scale used elsewhere in this index. R2 not reported anywhere in the paper. Paper also fits a smoking-cessation-rate vs. cigarette-price curve (one-phase decay model) using the breakpoint index, estimating a price of at least 37.36 yuan/pack would be needed to reduce mainland China's smoking prevalence to the Healthy China 2030 target of 20% -- out of HPT-index scope, not coded here. First China/CNY entry in the index.</t>
+        </is>
+      </c>
+    </row>
     <row r="377" ht="13" customHeight="1"/>
     <row r="378" ht="13" customHeight="1"/>
     <row r="379" ht="13" customHeight="1"/>

</xml_diff>

<commit_message>
Add Lin, Chen, & Song (2025) hotel demand HPT (3 rows, by hotel tier)
Peer-reviewed (Journal of Hospitality & Tourism Research). 3 hotel
types (economy/midscale/upscale) x 2 consumption situations (normal/
pandemic) -- coded as 3 rows (one per tier), averaging normal/
pandemic per tier where both exist, same collapsing rule used for
Goto2026. New distinct commodity strings per tier (economy/midscale/
upscale hotel room), separate from the existing plain "Hotel rooms"
entry used in an unrelated study. Demand measured as purchase
probability (Q0=100% in every condition), not consumption quantity --
flagged in notes as not comparable to Q0 elsewhere in the index.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL376"/>
+  <dimension ref="A1:AL379"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -72713,9 +72713,513 @@
         </is>
       </c>
     </row>
-    <row r="377" ht="13" customHeight="1"/>
-    <row r="378" ht="13" customHeight="1"/>
-    <row r="379" ht="13" customHeight="1"/>
+    <row r="377" ht="13" customHeight="1">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Lin2025-eco</t>
+        </is>
+      </c>
+      <c r="B377" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Journal of Hospitality &amp; Tourism Research</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>10.1177/10963480241271307</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/10963480241271307</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>Economy hotel room</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Leisure &amp; Entertainment</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N377" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="P377" t="n">
+        <v>274</v>
+      </c>
+      <c r="Q377" t="inlineStr">
+        <is>
+          <t>Chinese adults (online panel, Credamo)</t>
+        </is>
+      </c>
+      <c r="R377" t="n">
+        <v>36.46</v>
+      </c>
+      <c r="S377" t="n">
+        <v>13</v>
+      </c>
+      <c r="T377" t="n">
+        <v>0</v>
+      </c>
+      <c r="U377" t="n">
+        <v>1500</v>
+      </c>
+      <c r="V377" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="W377" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X377" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA377" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB377" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AE377" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AF377" t="inlineStr">
+        <is>
+          <t>Essential Value (EV=5.92); Omax (maximum expenditure, ¥158.0)</t>
+        </is>
+      </c>
+      <c r="AG377" t="n">
+        <v>0.000504</v>
+      </c>
+      <c r="AH377" t="inlineStr">
+        <is>
+          <t>100 (%, purchase probability -- not comparable to other studies' Q0)</t>
+        </is>
+      </c>
+      <c r="AJ377" t="n">
+        <v>495</v>
+      </c>
+      <c r="AK377" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AL377" t="inlineStr">
+        <is>
+          <t>Peer-reviewed (Journal of Hospitality &amp; Tourism Research, 2025). 3(hotel type) x 2(consumption situation: normal/pandemic) between-subjects HPT experiment, N=822 total valid responses across 6 roughly-equal experimental cells (exact per-cell N only in an online supplement not accessible here -- sample_size below is an estimate, total/3). Demand was measured as PURCHASE PROBABILITY (0-100%), not consumption quantity like the rest of this index -- Q0=100% in every condition (everyone would take a free hotel room with certainty), so Q0 here is not comparable to Q0 elsewhere in the dataset. No breakpoint reported anywhere (the paper's index set is R2/Q0/alpha/EV/Pmax/Omax, not the standard 5-index framework). Essential Value (EV) is this paper's central contribution but has no dedicated numeric column in this schema -- see below for EV alongside Omax. Group demand curves were fit to mean/aggregate data per condition, not per individual. This row: Economy hotels -- the pandemic did not significantly change the demand curve for this tier, so the paper reports one combined value (no averaging needed here).</t>
+        </is>
+      </c>
+    </row>
+    <row r="378" ht="13" customHeight="1">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Lin2025-mid</t>
+        </is>
+      </c>
+      <c r="B378" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Journal of Hospitality &amp; Tourism Research</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>10.1177/10963480241271307</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/10963480241271307</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>Midscale hotel room</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Leisure &amp; Entertainment</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N378" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="O378" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="P378" t="n">
+        <v>274</v>
+      </c>
+      <c r="Q378" t="inlineStr">
+        <is>
+          <t>Chinese adults (online panel, Credamo)</t>
+        </is>
+      </c>
+      <c r="R378" t="n">
+        <v>36.46</v>
+      </c>
+      <c r="S378" t="n">
+        <v>13</v>
+      </c>
+      <c r="T378" t="n">
+        <v>0</v>
+      </c>
+      <c r="U378" t="n">
+        <v>2250</v>
+      </c>
+      <c r="V378" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="W378" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X378" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y378" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z378" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA378" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB378" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC378" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD378" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AE378" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AF378" t="inlineStr">
+        <is>
+          <t>Essential Value (EV=9.13); Omax (maximum expenditure, ¥236.0)</t>
+        </is>
+      </c>
+      <c r="AG378" t="n">
+        <v>0.00038</v>
+      </c>
+      <c r="AH378" t="inlineStr">
+        <is>
+          <t>100 (%, purchase probability -- not comparable to other studies' Q0)</t>
+        </is>
+      </c>
+      <c r="AJ378" t="n">
+        <v>747</v>
+      </c>
+      <c r="AK378" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="AL378" t="inlineStr">
+        <is>
+          <t>Peer-reviewed (Journal of Hospitality &amp; Tourism Research, 2025). 3(hotel type) x 2(consumption situation: normal/pandemic) between-subjects HPT experiment, N=822 total valid responses across 6 roughly-equal experimental cells (exact per-cell N only in an online supplement not accessible here -- sample_size below is an estimate, total/3). Demand was measured as PURCHASE PROBABILITY (0-100%), not consumption quantity like the rest of this index -- Q0=100% in every condition (everyone would take a free hotel room with certainty), so Q0 here is not comparable to Q0 elsewhere in the dataset. No breakpoint reported anywhere (the paper's index set is R2/Q0/alpha/EV/Pmax/Omax, not the standard 5-index framework). Essential Value (EV) is this paper's central contribution but has no dedicated numeric column in this schema -- see below for EV alongside Omax. Group demand curves were fit to mean/aggregate data per condition, not per individual. This row: Midscale hotels -- averaged across Normal (R2=0.95, alpha=4.03e-4, EV=8.58, Pmax=702, Omax=222) and Pandemic (R2=0.96, alpha=3.57e-4, EV=9.68, Pmax=792, Omax=250) conditions, which the paper found significantly different (pandemic made demand more inelastic) -- averaging obscures that finding; see the paper for the real per-condition values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="379" ht="13" customHeight="1">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Lin2025-ups</t>
+        </is>
+      </c>
+      <c r="B379" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Journal of Hospitality &amp; Tourism Research</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>10.1177/10963480241271307</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/10963480241271307</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>Upscale hotel room</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Leisure &amp; Entertainment</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N379" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="O379" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="P379" t="n">
+        <v>274</v>
+      </c>
+      <c r="Q379" t="inlineStr">
+        <is>
+          <t>Chinese adults (online panel, Credamo)</t>
+        </is>
+      </c>
+      <c r="R379" t="n">
+        <v>36.46</v>
+      </c>
+      <c r="S379" t="n">
+        <v>13</v>
+      </c>
+      <c r="T379" t="n">
+        <v>0</v>
+      </c>
+      <c r="U379" t="n">
+        <v>3000</v>
+      </c>
+      <c r="V379" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="W379" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X379" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y379" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z379" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA379" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB379" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC379" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD379" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AE379" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AF379" t="inlineStr">
+        <is>
+          <t>Essential Value (EV=21.00); Omax (maximum expenditure, ¥503.5)</t>
+        </is>
+      </c>
+      <c r="AG379" t="n">
+        <v>0.000238</v>
+      </c>
+      <c r="AH379" t="inlineStr">
+        <is>
+          <t>100 (%, purchase probability -- not comparable to other studies' Q0)</t>
+        </is>
+      </c>
+      <c r="AJ379" t="n">
+        <v>1642.5</v>
+      </c>
+      <c r="AK379" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="AL379" t="inlineStr">
+        <is>
+          <t>Peer-reviewed (Journal of Hospitality &amp; Tourism Research, 2025). 3(hotel type) x 2(consumption situation: normal/pandemic) between-subjects HPT experiment, N=822 total valid responses across 6 roughly-equal experimental cells (exact per-cell N only in an online supplement not accessible here -- sample_size below is an estimate, total/3). Demand was measured as PURCHASE PROBABILITY (0-100%), not consumption quantity like the rest of this index -- Q0=100% in every condition (everyone would take a free hotel room with certainty), so Q0 here is not comparable to Q0 elsewhere in the dataset. No breakpoint reported anywhere (the paper's index set is R2/Q0/alpha/EV/Pmax/Omax, not the standard 5-index framework). Essential Value (EV) is this paper's central contribution but has no dedicated numeric column in this schema -- see below for EV alongside Omax. Group demand curves were fit to mean/aggregate data per condition, not per individual. This row: Upscale hotels -- averaged across Normal (R2=0.96, alpha=2.21e-4, EV=22.48, Pmax=1758, Omax=539) and Pandemic (R2=0.97, alpha=2.55e-4, EV=19.52, Pmax=1527, Omax=468) conditions, which the paper found significantly different (pandemic made demand more elastic) -- averaging obscures that finding; see the paper for the real per-condition values.</t>
+        </is>
+      </c>
+    </row>
     <row r="380" ht="13" customHeight="1"/>
     <row r="381" ht="13" customHeight="1"/>
     <row r="382" ht="13" customHeight="1"/>

</xml_diff>

<commit_message>
Add Tewogbola, Jacobs, & McDaniel (2023) HIV/COVID vaccine HPT (2 rows)
Self-authored (PI, PROMISE Labs Africa), medRxiv preprint. Vaccine
type (COVID-19/HIV) was within-subjects, so coded as 2 commodity rows
rather than averaged; country (Nigeria/USA) was between-subjects and
pooled per row using the paper's own cross-country aggregate values
(Figure 2a) -- this obscures a significant country x vaccine-type
interaction, flagged in notes. New "HIV vaccine" commodity, mapped to
Health & Prevention alongside the existing "COVID-19 vaccine". Price
is hospitalization-risk probability substituted for money, and Q0 is
purchase-probability rather than quantity -- both flagged as not
directly comparable to the rest of the index.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL379"/>
+  <dimension ref="A1:AL381"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -73220,8 +73220,322 @@
         </is>
       </c>
     </row>
-    <row r="380" ht="13" customHeight="1"/>
-    <row r="381" ht="13" customHeight="1"/>
+    <row r="380" ht="13" customHeight="1">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Tewogbola2023-covid</t>
+        </is>
+      </c>
+      <c r="B380" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>medRxiv (preprint)</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>10.1101/2023.07.24.23293101</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>https://www.medrxiv.org/content/10.1101/2023.07.24.23293101v1</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>COVID-19 vaccine</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t>Nigeria; United States</t>
+        </is>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>Multi-regional</t>
+        </is>
+      </c>
+      <c r="P380" t="n">
+        <v>109</v>
+      </c>
+      <c r="Q380" t="inlineStr">
+        <is>
+          <t>Mixed community sample (US MTurk workers; Nigerian social media-recruited adults)</t>
+        </is>
+      </c>
+      <c r="S380" t="n">
+        <v>11</v>
+      </c>
+      <c r="T380" t="n">
+        <v>0</v>
+      </c>
+      <c r="U380" t="n">
+        <v>1</v>
+      </c>
+      <c r="V380" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W380" t="inlineStr">
+        <is>
+          <t>Hursh &amp; Silberberg exponential model</t>
+        </is>
+      </c>
+      <c r="X380" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y380" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z380" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA380" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB380" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC380" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD380" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE380" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AH380" t="inlineStr">
+        <is>
+          <t>91.2 (%, purchase probability -- not comparable to other studies' Q0)</t>
+        </is>
+      </c>
+      <c r="AJ380" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="AK380" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AL380" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs and Justin T. McDaniel (SIU Carbondale). medRxiv preprint, not yet peer-reviewed. N=109 (65 Nigeria, 44 USA); vaccine type (COVID-19/HIV) was within-subjects (same participants rated both), country was between-subjects. Pooled across country here (using Figure 2a's own cross-country aggregate values) -- this obscures the paper's actual key finding, a significant country x vaccine-type interaction (Nigerian participants showed higher demand for the HIV vaccine than COVID-19; American participants showed the reverse); see the paper for the real per-country values. "Price" is hospitalization risk from the vaccine (0=no risk, 1=certain hospitalization), substituted for a monetary price -- lowest_price/highest_price represent that probability scale, not currency. Q0 is measured as purchase-probability (0-100%), not consumption quantity -- not comparable to Q0 elsewhere in this index. No single aggregate alpha value is stated in the text (only shown per-individual for the 10 best-fitting curves per vaccine in Table 1), so mean_alpha is left blank rather than guessed. No breakpoint or essential value reported, despite essential value being discussed conceptually in the introduction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="381" ht="13" customHeight="1">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Tewogbola2023-hiv</t>
+        </is>
+      </c>
+      <c r="B381" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>medRxiv (preprint)</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>10.1101/2023.07.24.23293101</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>https://www.medrxiv.org/content/10.1101/2023.07.24.23293101v1</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Preprint</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N381" t="inlineStr">
+        <is>
+          <t>Nigeria; United States</t>
+        </is>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>Multi-regional</t>
+        </is>
+      </c>
+      <c r="P381" t="n">
+        <v>109</v>
+      </c>
+      <c r="Q381" t="inlineStr">
+        <is>
+          <t>Mixed community sample (US MTurk workers; Nigerian social media-recruited adults)</t>
+        </is>
+      </c>
+      <c r="S381" t="n">
+        <v>11</v>
+      </c>
+      <c r="T381" t="n">
+        <v>0</v>
+      </c>
+      <c r="U381" t="n">
+        <v>1</v>
+      </c>
+      <c r="V381" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W381" t="inlineStr">
+        <is>
+          <t>Hursh &amp; Silberberg exponential model</t>
+        </is>
+      </c>
+      <c r="X381" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y381" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z381" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA381" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB381" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AC381" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD381" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE381" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AH381" t="inlineStr">
+        <is>
+          <t>92.4 (%, purchase probability -- not comparable to other studies' Q0)</t>
+        </is>
+      </c>
+      <c r="AJ381" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AK381" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="AL381" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs and Justin T. McDaniel (SIU Carbondale). medRxiv preprint, not yet peer-reviewed. N=109 (65 Nigeria, 44 USA); vaccine type (COVID-19/HIV) was within-subjects (same participants rated both), country was between-subjects. Pooled across country here (using Figure 2a's own cross-country aggregate values) -- this obscures the paper's actual key finding, a significant country x vaccine-type interaction (Nigerian participants showed higher demand for the HIV vaccine than COVID-19; American participants showed the reverse); see the paper for the real per-country values. "Price" is hospitalization risk from the vaccine (0=no risk, 1=certain hospitalization), substituted for a monetary price -- lowest_price/highest_price represent that probability scale, not currency. Q0 is measured as purchase-probability (0-100%), not consumption quantity -- not comparable to Q0 elsewhere in this index. No single aggregate alpha value is stated in the text (only shown per-individual for the 10 best-fitting curves per vaccine in Table 1), so mean_alpha is left blank rather than guessed. No breakpoint or essential value reported, despite essential value being discussed conceptually in the introduction.</t>
+        </is>
+      </c>
+    </row>
     <row r="382" ht="13" customHeight="1"/>
     <row r="383" ht="13" customHeight="1"/>
     <row r="384" ht="13" customHeight="1"/>

</xml_diff>

<commit_message>
Add Tewogbola et al. (2025) "Beyond the jab" HIV vaccine HPT (10 rows)
Self-authored (PI, PROMISE Labs Africa), peer-reviewed (J Exp Anal
Behav). Experiment 1 (administration mode x dosage) collapsed to one
row since the paper found those manipulations had minimal effect on
demand; Experiment 2 (HIV vaccine bundled with 9 other health
commodities) coded as 9 separate rows straight from the paper's own
Table 5. Study IDs use the Tewogbola2025-hiv- prefix to match the
existing Tewogbola2025-ins/-mil convention.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL381"/>
+  <dimension ref="A1:AL391"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -73536,16 +73536,1656 @@
         </is>
       </c>
     </row>
-    <row r="382" ht="13" customHeight="1"/>
-    <row r="383" ht="13" customHeight="1"/>
-    <row r="384" ht="13" customHeight="1"/>
-    <row r="385" ht="13" customHeight="1"/>
-    <row r="386" ht="13" customHeight="1"/>
-    <row r="387" ht="13" customHeight="1"/>
-    <row r="388" ht="13" customHeight="1"/>
-    <row r="389" ht="13" customHeight="1"/>
-    <row r="390" ht="13" customHeight="1"/>
-    <row r="391" ht="13" customHeight="1"/>
+    <row r="382" ht="13" customHeight="1">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-e1</t>
+        </is>
+      </c>
+      <c r="B382" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N382" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O382" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P382" t="n">
+        <v>285</v>
+      </c>
+      <c r="Q382" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R382" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S382" t="n">
+        <v>15</v>
+      </c>
+      <c r="T382" t="n">
+        <v>0</v>
+      </c>
+      <c r="U382" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V382" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W382" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X382" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA382" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD382" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE382" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG382" t="n">
+        <v>6.397e-06</v>
+      </c>
+      <c r="AH382" t="n">
+        <v>70.33</v>
+      </c>
+      <c r="AI382" t="n">
+        <v>522.33</v>
+      </c>
+      <c r="AJ382" t="n">
+        <v>434.16</v>
+      </c>
+      <c r="AK382" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="AL382" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 1 (N=285), participants randomized to 9 groups crossing vaccine administration mode (oral/mucosal/subcutaneous) x perceived dosage (one dose/two doses/annual dose). The paper's key finding was that these vaccine-characteristic manipulations had minimal effect on demand (regression R²=.007 for Q0, R²=.001 for log alpha, both ns after Bonferroni correction -- see Table 3); individual factors (injection drug use history, experienced racial discrimination, prior vaccine uptake, trust in science/government, low household income) were the significant predictors instead. Because condition had so little effect, and the paper did not report a single pooled aggregate across all 9 cells (only the 3 mode-marginal and 3 dosage-marginal aggregates in Table 2, which are two different collapses of the same 285 participants), this row is the simple mean of those 6 marginal Q0/alpha/Pmax/breakpoint/R² values as an approximation of the overall aggregate -- see Table 2 for the real per-condition breakdown. Experiment 2 (bundling) is entered as 9 separate rows below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="383" ht="13" customHeight="1">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-prep</t>
+        </is>
+      </c>
+      <c r="B383" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N383" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P383" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q383" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R383" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S383" t="n">
+        <v>15</v>
+      </c>
+      <c r="T383" t="n">
+        <v>0</v>
+      </c>
+      <c r="U383" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V383" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W383" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X383" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA383" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD383" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE383" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG383" t="n">
+        <v>6.93e-06</v>
+      </c>
+      <c r="AH383" t="n">
+        <v>71.51000000000001</v>
+      </c>
+      <c r="AI383" t="n">
+        <v>621</v>
+      </c>
+      <c r="AJ383" t="n">
+        <v>380.66</v>
+      </c>
+      <c r="AK383" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="AL383" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=24 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with PrEP, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2). This is the reference condition in Table 6's regression models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="384" ht="13" customHeight="1">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-hivtest</t>
+        </is>
+      </c>
+      <c r="B384" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N384" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P384" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q384" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R384" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S384" t="n">
+        <v>15</v>
+      </c>
+      <c r="T384" t="n">
+        <v>0</v>
+      </c>
+      <c r="U384" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V384" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W384" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X384" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y384" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z384" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA384" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB384" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC384" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD384" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE384" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG384" t="n">
+        <v>8.16e-06</v>
+      </c>
+      <c r="AH384" t="n">
+        <v>81.62</v>
+      </c>
+      <c r="AI384" t="n">
+        <v>462</v>
+      </c>
+      <c r="AJ384" t="n">
+        <v>261.83</v>
+      </c>
+      <c r="AK384" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AL384" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=26 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with an HIV test kit, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="385" ht="13" customHeight="1">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-condoms</t>
+        </is>
+      </c>
+      <c r="B385" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N385" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P385" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q385" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R385" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S385" t="n">
+        <v>15</v>
+      </c>
+      <c r="T385" t="n">
+        <v>0</v>
+      </c>
+      <c r="U385" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V385" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W385" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X385" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA385" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD385" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE385" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG385" t="n">
+        <v>5.2e-06</v>
+      </c>
+      <c r="AH385" t="n">
+        <v>68.45999999999999</v>
+      </c>
+      <c r="AI385" t="n">
+        <v>502</v>
+      </c>
+      <c r="AJ385" t="n">
+        <v>530.03</v>
+      </c>
+      <c r="AK385" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AL385" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=27 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with condoms, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2). Log alpha differed significantly from the PrEP-bundle reference before correction (β=0.91, p=.02) -- higher price sensitivity, interpreted as possible perceived redundancy with condoms as HIV prevention -- but not after Bonferroni correction (adjusted p&lt;.005; see Table 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="386" ht="13" customHeight="1">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-covid</t>
+        </is>
+      </c>
+      <c r="B386" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N386" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O386" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P386" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q386" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R386" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S386" t="n">
+        <v>15</v>
+      </c>
+      <c r="T386" t="n">
+        <v>0</v>
+      </c>
+      <c r="U386" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V386" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W386" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X386" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y386" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z386" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA386" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB386" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC386" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD386" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE386" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG386" t="n">
+        <v>7.849999999999999e-06</v>
+      </c>
+      <c r="AH386" t="n">
+        <v>76.73999999999999</v>
+      </c>
+      <c r="AI386" t="n">
+        <v>504</v>
+      </c>
+      <c r="AJ386" t="n">
+        <v>313.27</v>
+      </c>
+      <c r="AK386" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="AL386" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=27 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with a COVID-19 vaccine, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="387" ht="13" customHeight="1">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-flu</t>
+        </is>
+      </c>
+      <c r="B387" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N387" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P387" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q387" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R387" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S387" t="n">
+        <v>15</v>
+      </c>
+      <c r="T387" t="n">
+        <v>0</v>
+      </c>
+      <c r="U387" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V387" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W387" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X387" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y387" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z387" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA387" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB387" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC387" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD387" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE387" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG387" t="n">
+        <v>5.56e-06</v>
+      </c>
+      <c r="AH387" t="n">
+        <v>65.59</v>
+      </c>
+      <c r="AI387" t="n">
+        <v>573</v>
+      </c>
+      <c r="AJ387" t="n">
+        <v>517.85</v>
+      </c>
+      <c r="AK387" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AL387" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=27 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with a flu vaccine, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="388" ht="13" customHeight="1">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-hpv</t>
+        </is>
+      </c>
+      <c r="B388" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N388" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P388" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q388" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R388" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S388" t="n">
+        <v>15</v>
+      </c>
+      <c r="T388" t="n">
+        <v>0</v>
+      </c>
+      <c r="U388" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V388" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W388" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X388" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y388" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z388" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA388" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB388" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC388" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD388" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE388" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG388" t="n">
+        <v>5.77e-06</v>
+      </c>
+      <c r="AH388" t="n">
+        <v>81.44</v>
+      </c>
+      <c r="AI388" t="n">
+        <v>501</v>
+      </c>
+      <c r="AJ388" t="n">
+        <v>401.66</v>
+      </c>
+      <c r="AK388" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AL388" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=26 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with an HPV vaccine, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="389" ht="13" customHeight="1">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-dental</t>
+        </is>
+      </c>
+      <c r="B389" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N389" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P389" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q389" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R389" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S389" t="n">
+        <v>15</v>
+      </c>
+      <c r="T389" t="n">
+        <v>0</v>
+      </c>
+      <c r="U389" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V389" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W389" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X389" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y389" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z389" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA389" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB389" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC389" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD389" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE389" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG389" t="n">
+        <v>4.65e-06</v>
+      </c>
+      <c r="AH389" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="AI389" t="n">
+        <v>763</v>
+      </c>
+      <c r="AJ389" t="n">
+        <v>595.51</v>
+      </c>
+      <c r="AK389" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AL389" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=28 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with a free dental examination, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2). Log alpha differed significantly from the PrEP-bundle reference before correction (β=0.78, p=.04) -- higher price sensitivity, interpreted as possible perceived low relevance of dental care to HIV prevention -- but not after Bonferroni correction (adjusted p&lt;.005; see Table 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="390" ht="13" customHeight="1">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-eye</t>
+        </is>
+      </c>
+      <c r="B390" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N390" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O390" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P390" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q390" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R390" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S390" t="n">
+        <v>15</v>
+      </c>
+      <c r="T390" t="n">
+        <v>0</v>
+      </c>
+      <c r="U390" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V390" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W390" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X390" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA390" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD390" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE390" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG390" t="n">
+        <v>7.82e-06</v>
+      </c>
+      <c r="AH390" t="n">
+        <v>81.52</v>
+      </c>
+      <c r="AI390" t="n">
+        <v>458</v>
+      </c>
+      <c r="AJ390" t="n">
+        <v>296.15</v>
+      </c>
+      <c r="AK390" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="AL390" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=25 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with a free eye examination, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="391" ht="13" customHeight="1">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Tewogbola2025-hiv-mhc</t>
+        </is>
+      </c>
+      <c r="B391" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Journal of the Experimental Analysis of Behavior</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jeab.70038</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>HIV vaccine</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Health &amp; Prevention</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>Between-subjects</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N391" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>North America</t>
+        </is>
+      </c>
+      <c r="P391" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q391" t="inlineStr">
+        <is>
+          <t>Sexual and gender minority adults (Reddit- and LGBTQ+ community organization-recruited)</t>
+        </is>
+      </c>
+      <c r="R391" t="n">
+        <v>29.37</v>
+      </c>
+      <c r="S391" t="n">
+        <v>15</v>
+      </c>
+      <c r="T391" t="n">
+        <v>0</v>
+      </c>
+      <c r="U391" t="n">
+        <v>2000</v>
+      </c>
+      <c r="V391" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="W391" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X391" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="Y391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA391" t="inlineStr">
+        <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AB391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AD391" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE391" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AG391" t="n">
+        <v>4.48e-06</v>
+      </c>
+      <c r="AH391" t="n">
+        <v>77.77</v>
+      </c>
+      <c r="AI391" t="n">
+        <v>603</v>
+      </c>
+      <c r="AJ391" t="n">
+        <v>542.0700000000001</v>
+      </c>
+      <c r="AK391" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="AL391" t="inlineStr">
+        <is>
+          <t>Self-authored by the PI (PROMISE Labs Africa), with Eric A. Jacobs, Yueh-Ting Lee, and Ryan N. Redner (SIU Carbondale School of Psychological and Behavioral Sciences), Justin T. McDaniel (SIU School of Health Sciences), and Jebaraj Asirvatham (SIU School of Agricultural Sciences). Peer-reviewed (Journal of the Experimental Analysis of Behavior, 2025). Open-access status not confirmed -- no CC license visible on the article pages reviewed here, so marked No pending verification. Both experiments used the same 393 recruited sexual/gender-minority participants (Reddit + LGBTQ+ community organizations, U.S., aged 19+); Experiment 1 retained N=285 after exclusions, Experiment 2 retained N=236 (all Experiment-1 completers were invited into Experiment 2). 15 price points, $0-$2,000, VAS-slider purchase-likelihood task adapted from Hursh et al. (2020). This row: Experiment 2 (bundle-condition n=25 of N=236 total; Table 4's 9 per-bundle n's sum to 235, one short of the stated 236 -- discrepancy in the source, not corrected here), demand for a hypothetical HIV vaccine bundled with mental health counseling, values from Table 5. Bundling effects were subtle overall across the 9 conditions (Q0 R²=.016, log alpha R²=.104 -- see Table 6), smaller than the effect of individual factors (Q0 R²=.40, log alpha R²=.32 -- see Table 6 Model 2).</t>
+        </is>
+      </c>
+    </row>
     <row r="392" ht="13" customHeight="1"/>
     <row r="393" ht="13" customHeight="1"/>
     <row r="394" ht="13" customHeight="1"/>

</xml_diff>

<commit_message>
Add Acuff et al. (2022) six-country Internet demand HPT (1 pooled row)
Not self-authored -- independent multi-site group (Memphis lead, with
Argentina/Australia/India/Malaysia/UK co-authors), peer-reviewed (Exp
Clin Psychopharmacol). Commodity is "Internet Access" to match the
existing Broadbent2015 term, since this study explicitly uses the
same Internet Purchase Task. N-weighted pooled across all six
countries from Table 1's per-country means, following the same
collapse convention used for Tewogbola2023 -- notes flag that this
obscures the paper's actual key finding of significant cross-country
and GDP-group differences, with a pointer to Tables 1 and 3 for the
real breakdown. Elasticity mapped to alpha and Intensity to Q0 per
the paper's own terminology; k=2.08 and R2=.97 taken directly from
the text.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPT Resource Index.xlsx
+++ b/HPT Resource Index.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL391"/>
+  <dimension ref="A1:AL392"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="12.33203125" customWidth="1" min="1" max="1"/>
@@ -75186,7 +75186,171 @@
         </is>
       </c>
     </row>
-    <row r="392" ht="13" customHeight="1"/>
+    <row r="392" ht="13" customHeight="1">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Acuff2022-int</t>
+        </is>
+      </c>
+      <c r="B392" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Experimental and Clinical Psychopharmacology</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>10.1037/pha0000459</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1037/pha0000459</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Peer-Reviewed</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>Internet Access</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Leisure &amp; Entertainment</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>Cross-sectional</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N392" t="inlineStr">
+        <is>
+          <t>United States; Argentina; Australia; Malaysia; United Kingdom; India</t>
+        </is>
+      </c>
+      <c r="O392" t="inlineStr">
+        <is>
+          <t>Multi-regional</t>
+        </is>
+      </c>
+      <c r="P392" t="n">
+        <v>1406</v>
+      </c>
+      <c r="Q392" t="inlineStr">
+        <is>
+          <t>College students (six-country sample)</t>
+        </is>
+      </c>
+      <c r="R392" t="n">
+        <v>20.92</v>
+      </c>
+      <c r="S392" t="n">
+        <v>25</v>
+      </c>
+      <c r="T392" t="n">
+        <v>0</v>
+      </c>
+      <c r="U392" t="n">
+        <v>100</v>
+      </c>
+      <c r="V392" t="inlineStr">
+        <is>
+          <t>USD (PPP-equivalized across countries)</t>
+        </is>
+      </c>
+      <c r="W392" t="inlineStr">
+        <is>
+          <t>Koffarnus et al. exponentiated model</t>
+        </is>
+      </c>
+      <c r="X392" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="Y392" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Z392" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AA392" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB392" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AC392" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AD392" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE392" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AF392" t="inlineStr">
+        <is>
+          <t>Omax (maximum expenditure, $30.19 PPP-USD, N-weighted across countries)</t>
+        </is>
+      </c>
+      <c r="AG392" t="n">
+        <v>0.01875</v>
+      </c>
+      <c r="AH392" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="AI392" t="n">
+        <v>18.71</v>
+      </c>
+      <c r="AK392" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="AL392" t="inlineStr">
+        <is>
+          <t>Not self-authored -- independent multi-site group (University of Memphis lead, with co-authors in Argentina, Australia, India, Malaysia, and the UK). Peer-reviewed (Experimental and Clinical Psychopharmacology); published online first 2021-04-29, print issue Vol. 30 No. 5 (2022) -- coded here as 2022 to match the print volume/issue. Open-access status not confirmed -- no CC license visible on the article pages reviewed, marked No pending verification. Cross-sectional, six-country college-student sample (United States n=217, Argentina n=300, Australia n=254, Malaysia n=323, United Kingdom n=173, India n=153 -- these six Table 1 n's sum to 1,420, slightly above the paper's stated total N=1,406; the paper's own footnote notes per-index exclusions differ slightly, e.g. 47 participants dropped from elasticity only for Stein's-criteria inconsistency, so per-index/per-country n's are not perfectly uniform). Prices were set in USD ($0-$100, 25 escalating points above the free/$0 anchor) then multiplied by each country's Purchasing Power Parity index (Argentina 13.56 pesos/USD; Australia 1.44 AUD/USD; Malaysia 1.46 Ringgit/USD; UK 0.7 GBP/USD; India 18.04 Rupees/USD, as of the 2018 study launch) so consumption is comparable at equivalent real purchasing power -- currency is nominally USD but PPP-equivalized, not raw local currency. Q0/Breakpoint/Omax/Elasticity here are the simple N-weighted mean of Table 1's six country-level means (weights = each country's Table 1 n) -- a considerable simplification, since the paper's actual key finding is significant CROSS-COUNTRY differences on nearly every index (all F/chi-square tests in Table 1 significant at p&lt;.02 or lower) and significant differences by GDP-per-capita group, sex at birth, and income (Table 3) -- see Table 1 (by country) and Table 3 (by GDP group/sex/income) for the real breakdown, not reproduced as separate rows here. Elasticity mapped to this index's alpha field and Intensity mapped to Q0 -- both are the paper's own terms for the exponentiated-model parameters (Koffarnus et al., 2015). No Pmax reported (only Intensity/Breakpoint/Omax/Elasticity used); Omax entered as text under Other since this schema's Pmax field is a different index (price of max expenditure, not reported here) -- Omax value above is also the N-weighted pooled mean. k=2.08, calculated empirically per Koffarnus et al. (2015) from the log10-transformed consumption range, not fit per individual. R2: participant-level full-sample mean R2=.94 (median .96); aggregate full-sample R2=.97 (used as mean_r2 here); country-level aggregate R2 ranged .95-.99 (not broken out per country in this row). Demand indices also feed a larger structural equation model relating Internet demand, delay discounting, and alternative reinforcement to harmful Internet use, smartphone addiction, online gaming, and Internet sexual behavior (Figure 3) -- out of this index's HPT-demand scope, not coded here.</t>
+        </is>
+      </c>
+    </row>
     <row r="393" ht="13" customHeight="1"/>
     <row r="394" ht="13" customHeight="1"/>
     <row r="395" ht="13" customHeight="1"/>

</xml_diff>